<commit_message>
Update references in validation checks
Add references to updated DCEG clause 2.4.4 in checks 122_0059 and 122_0060
</commit_message>
<xml_diff>
--- a/S158_122/1.0.0/S-158_122_1_0_0_20260323.xlsx
+++ b/S158_122/1.0.0/S-158_122_1_0_0_20260323.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\work\git\S-122-Product-Specification-Development\S158_122\1.0.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F4898AD-298B-4365-A0BF-3294727D115E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0B9FF0A-A124-49E5-9CED-8840635E3EAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="28110" windowHeight="18240" tabRatio="647" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="319">
   <si>
     <t>Document Number</t>
   </si>
@@ -1037,6 +1037,9 @@
   </si>
   <si>
     <t>For each attribute binding listed in in DCEG clause 2.4 as not nillable AND which is not populated</t>
+  </si>
+  <si>
+    <t>2.4.4</t>
   </si>
 </sst>
 </file>
@@ -4539,9 +4542,11 @@
         <v>288</v>
       </c>
       <c r="G60" s="57" t="s">
-        <v>166</v>
-      </c>
-      <c r="H60" s="85"/>
+        <v>68</v>
+      </c>
+      <c r="H60" s="85" t="s">
+        <v>318</v>
+      </c>
       <c r="I60" s="46" t="s">
         <v>26</v>
       </c>
@@ -4574,9 +4579,11 @@
         <v>292</v>
       </c>
       <c r="G61" s="57" t="s">
-        <v>166</v>
-      </c>
-      <c r="H61" s="85"/>
+        <v>68</v>
+      </c>
+      <c r="H61" s="85" t="s">
+        <v>318</v>
+      </c>
       <c r="I61" s="46" t="s">
         <v>26</v>
       </c>

</xml_diff>